<commit_message>
Capture first five Texas CRDs via record-page search
FINRA, SEC IAPD and FDIC remain unreachable on a third reachability
test, so the BrokerCheck/IAPD lookups were run through search of those
record pages instead. Texas went from zero CRDs to five.

- Jim Brown (Texas Capital) CRD 1215292 — registered 05/03/2025, joined
  April 2025 from 20 years at Wells Fargo Private Bank as a Senior
  Private Wealth Portfolio Manager. Now the strongest Texas target.
- Laurie Wieters (Frost) CRD 1460584
- Ashley Ferguson (Frost) CRD 5667123
- Michael Hanson (Prosperity) CRD 2750146, ambiguous against 5417580
- Ronald Folwell (Woodforest) CRD 2128911 — "not currently registered as
  a broker" is consistent with his corporate-RIA role, not retirement

New CRD column on the Texas Advisors tab. None are verified against an
actual report.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012NtTkX4kFFRh2WeKuPwqNf
</commit_message>
<xml_diff>
--- a/texas-banks-wealth-management.xlsx
+++ b/texas-banks-wealth-management.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Tier 2 - Out of State" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Texas Advisors'!$A$4:$I$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Texas Advisors'!$A$4:$J$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +74,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -119,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,6 +145,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -504,7 +516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A59"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -524,7 +536,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -560,7 +571,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
@@ -596,7 +606,6 @@
         </is>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -632,7 +641,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
@@ -675,38 +683,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
-    <row r="29"/>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -718,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I45"/>
+  <dimension ref="A1:J45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -730,6 +706,7 @@
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="72" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -742,7 +719,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>36 named people across 9 banks. NO CRD captured for any Texas advisor and no registration verified — FINRA was unreachable. Run BrokerCheck before calling.</t>
+          <t>36 named people across 9 banks. 5 CRDs captured 2026-09-13 via search of FINRA/SEC records — FINRA itself is still unreachable, so NONE are verified against an actual report. Run BrokerCheck before calling.</t>
         </is>
       </c>
     </row>
@@ -790,6 +767,11 @@
       <c r="I4" s="6" t="inlineStr">
         <is>
           <t>Source URL</t>
+        </is>
+      </c>
+      <c r="J4" s="11" t="inlineStr">
+        <is>
+          <t>CRD (search-derived, UNVERIFIED)</t>
         </is>
       </c>
     </row>
@@ -1176,7 +1158,12 @@
       </c>
       <c r="I13" s="7" t="inlineStr">
         <is>
-          <t>https://www.prosperitybankusa.com/prosperityprivate-investments-bios/</t>
+          <t>https://www.prosperitybankusa.com/prosperityprivate-investments-bios/ | https://adviserinfo.sec.gov/individual/summary/2750146</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>2750146 (likely) — JOHN MICHAEL HANSON, Investment Adviser at Raymond James Financial Services Advisors. AMBIGUOUS: a separate MICHAEL D HANSON exists at CRD 5417580. Confirm which before use.</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1319,12 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>https://www.raymondjames.com/woodforestadvisors/about-us</t>
+          <t>https://www.raymondjames.com/woodforestadvisors/about-us | https://files.brokercheck.finra.org/individual/individual_2128911.pdf</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>2128911 — 'Ronald Lee Folwell Jr.' NOT CURRENTLY REGISTERED AS A BROKER. Consistent with his Woodforest role: he joined as a CORPORATE RIA-affiliated advisor, so he would sit on IAPD rather than BrokerCheck. Do not read this as retired. Career: began 1991 at Ameriprise (23 yrs), United Capital from 2014, Woodforest Aug 2024.</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1476,12 @@
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>https://texascapitalbank.com/private-bank/meet-our-advisors</t>
+          <t>https://texascapitalbank.com/private-bank/meet-our-advisors | https://reports.adviserinfo.sec.gov/reports/individual/individual_1215292.pdf</t>
+        </is>
+      </c>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>1215292 — JAMES MARCUS BROWN. Registered with Texas Capital Bank Private Wealth Advisors (firm CRD 298422) as of 05/03/2025. Joined April 2025 after 20 years at Wells Fargo Private Bank as Senior Private Wealth Portfolio Manager.</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1824,12 @@
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>https://www.frostbank.com/personal/investments/trust-estate-planning</t>
+          <t>https://www.frostbank.com/personal/investments/trust-estate-planning | https://smartadvisormatch.com/advisor-network/texas/laurie-wieters-1460584</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>1460584 — 39 years in the industry, Series 63 and 66, with Frost Investment Services since 2017; four decades across Frost Brokerage Services and Frost Bank.</t>
         </is>
       </c>
     </row>
@@ -1866,7 +1868,12 @@
       <c r="H31" s="7" t="inlineStr"/>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>https://www.frostbank.com/personal/investments/trust-estate-planning</t>
+          <t>https://www.frostbank.com/personal/investments/trust-estate-planning | https://smartadvisormatch.com/advisor-network/texas/ashley-ferguson-5667123</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>5667123 — prior Frost Brokerage Services, Frost National Bank, Frost Investment Services.</t>
         </is>
       </c>
     </row>
@@ -2237,6 +2244,7 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
@@ -2276,7 +2284,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I40"/>
+  <autoFilter ref="A4:J40"/>
   <mergeCells count="1">
     <mergeCell ref="A45:I45"/>
   </mergeCells>

</xml_diff>